<commit_message>
clienti: pagina e download solo per admin; commodities: LBS=F delistato → LBR=F
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Files/COMMODITIES.xlsx
+++ b/Files/COMMODITIES.xlsx
@@ -1014,12 +1014,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>LBS=F</t>
+          <t>LBR=F</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Random Length Lumber Futures</t>
+          <t>Lumber Futures</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">

</xml_diff>